<commit_message>
- Add some new files
</commit_message>
<xml_diff>
--- a/brilliantearth_rings/product_data.xlsx
+++ b/brilliantearth_rings/product_data.xlsx
@@ -425,30 +425,1025 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Product Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Image Links</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Video Link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Petite Lab Diamond Tube Ring</t>
+          <t>/Ballad-Half-Coverage-Diamond-Ring-(1/6-ct.-tw.)-White-Gold-BE2D1823</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/D8/BE2D629LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/BD/BE2D629LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/95/BE2D629LC_yellow_ms_zi.png</t>
+          <t>Ballad Half Coverage Diamond Ring (1/6 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/5F/BE2D1823_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/8B/BE2D1823_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/BN/BE2D1823E_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/75/BE2D1823_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/2A/BE2D1823_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>/Nouveau-Diamond-Ring-White-Gold-BE2D2359</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Nouveau Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/D8/BE2D2359_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/5F/BE2D2359_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/20/BE2D2359_white_additional1.jpeg, https://image.brilliantearth.com/media/product_images/71/BE2D2359_white_02.jpg, https://image.brilliantearth.com/media/product_images/T8/BE2D2359_white_hand_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/9280ce70-8718-4319-9e49-abecb31c67c1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>/Matte-Hammered-Petite-Comfort-Fit-Wedding-Ring-Gold-BE299MH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Matte Hammered Petite Comfort Fit Wedding Ring</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/J0/BE299MH_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE299MH_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/DT/BE299MH_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_images/ER/BE299MH_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/3C/BE299MH_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/0b514589-c8b9-425f-9f18-c34f895c60bf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>/Jardiniere-Diamond-Ring-Gold-BE2D835</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Jardiniere Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/CD/BE2D835_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/PJ/BE2D835-18KY_2.jpg, https://image.brilliantearth.com/media/product_images/76/BE2D835-18KY_3.jpg, https://image.brilliantearth.com/media/product_new_images/52/BE2D835_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/48/BE2D835_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/E5/BE2D835_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/78d6962e-0b2f-418b-9d24-ea42837fdf1e</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>/Luxe-Winding-Willow-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE2564LD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Luxe Winding Willow Diamond Ring (1/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/90/BE2564LD_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/04/BE2564LD_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/E4/BE2564LD-18KW.jpg, https://image.brilliantearth.com/media/product_images/3H/BE2564LD_white_side.jpg, https://image.brilliantearth.com/media/product_images/42/BE2564LD_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/92/BE2564LD_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/8fd59de9-323f-46d6-820b-fcef0eeb7748</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>/Petite-Shared-Prong-Three-Quarter-Coverage-Diamond-Ring-(3/8-ct.-tw.)-White-Gold-BE2PD28R15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Petite Shared Prong Three-Quarter Coverage Diamond Ring (3/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/3D/BE2PD28R15_white_top.jpg, https://image.brilliantearth.com/media/product_images/UH/BE2PD28R15-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FI/BE2PD28R15_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/4D/BE2PD28R15_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/65/BE2PD28R15_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/60cab62e-85bb-4423-8f3f-9a7b5126fccb</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>/Riviera-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Gold-BE2DR200ELC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Riviera Eternity Lab Diamond Ring (2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/D1/BE2DR200ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/A8/BE2DR200ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A7/BE2DR200ELC_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>/Versailles-Eternity-Lab-Diamond-Ring-(3/4-ct.-tw.)-Gold-BE2D1792LC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Versailles Eternity Lab Diamond Ring (3/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/96/BE2D1792_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/NE/BE2D1792-yellow_019.jpg, https://image.brilliantearth.com/media/product_new_images/E6/BE2D1792_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/64/BE2D1792_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/87e958c6-e357-430a-a2ea-581c5c3ebf07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>/Sienna-Eternity-Lab-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M3420ETLC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sienna Eternity Lab Diamond Ring (7/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/70/BE2M3420ET_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2M3420ETLC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/KP/BE2M3420-BE2M3420ET-BE2M3420H.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2M3420ET_white_side1.jpg, https://image.brilliantearth.com/media/product_images/DQ/BE2M3420ET_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/18/BE2M3420ET_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/2a84a988-a1cc-43f8-bb15-4ed049e33998</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>/Luxe-Tiara-Eternity-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D147E</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>18K White Gold
+            Luxe Tiara Eternity Diamond Ring (1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/A8/BE2D147E_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/AA/BE2D147E_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/7L/BE2D147E_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/DA/BE2D147E_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/6C/BE2D147E_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>/Riviera-Eternity-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2DR200E</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Riviera Eternity Diamond Ring (2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/9A/BE2DR200ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/9F/BE2DR200ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/78/BE2DR200ELC_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>/Whisper-Eternity-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE266E</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Whisper Eternity Diamond Ring (1/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/8C/BE266E_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/80/BE266E_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/FW/BE266E_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/84/BE266E_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/88/BE266E_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/f47739af-c394-4d3d-9c27-88895be403d6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>/Flair-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D1938</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Flair Diamond Ring (1/3 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/85/BE2D1938_white_top.jpg, https://image.brilliantearth.com/media/product_images/2V/BE2D1938.jpeg, https://image.brilliantearth.com/media/product_images/NW/BE2D1938_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/00/BE2D1938_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D7/BE2D1938_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/32238343-5dbf-4d21-a6f9-0dadece8c4ff</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>/Monaco-Diamond-Ring-(3/4-ct.-tw.)-White-Gold-BE2D829</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Monaco Diamond Ring (3/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/35/BE2D829_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/D3/BE2D829_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/W2/BE2D829_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/CC/BE2D829_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/DC/BE2D829_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>/Ellora-Half-Coverage-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M2811</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ellora Half Coverage Diamond Ring (7/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/06/BE2M2811_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/0D/BE2M2811_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/D2/BE2M2811_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/8D/BE2M2811_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/d4489832-4a72-41f8-892c-e0f44d0d3ec1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>/Curved-Versailles-Diamond-Ring-White-Gold-BE2D7422</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Curved Versailles Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/AC/BE2D7422_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/02/BE2D7422_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VK/BE2D7422_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>/Entwined-Diamond-Contour-Ring-(1/5-ct.-tw.)-Rose-Gold-BE2D1816</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Entwined Diamond Contour Ring (1/5 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/B3/BE2D1816_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/35/BE2D1816_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E7/BE2D1816_rose_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>/Sia-Half-Coverage-Lab-Diamond-Ring-(1/8-ct.-tw.)-Gold-BE2D2118PLC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sia Half Coverage Lab Diamond Ring (1/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/37/BE2D2118P_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/9C/BE2D2118P-yellow_2.jpg, https://image.brilliantearth.com/media/product_images/J2/BE2D2118P-yellow_4.jpg, https://image.brilliantearth.com/media/product_new_images/C9/BE2D2118P_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE2D2118P_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>/Chevron-Ring-Gold-BE2119</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chevron Ring</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/55/BE2119_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/50/BE2119_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/U6/YG2.jpg, https://image.brilliantearth.com/media/product_new_images/D0/BE2119_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/26bc93b2-094f-4a94-98f3-c942a4ef09eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>/Curved-Versailles-Lab-Diamond-Ring-White-Gold-BE2D7422LC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Curved Versailles Lab Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/AC/BE2D7422_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/02/BE2D7422_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VK/BE2D7422_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>/Gemma-Baguette-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D084B</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gemma Baguette Diamond Ring (1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/A6/BE2D084B_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/5A/BE2D084B_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/3F/BE2D084B_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/7R/BE2D084B_yellow_side.jpeg, https://image.brilliantearth.com/media/product_new_images/FD/BE2D084B_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>/Imogen-Pear-Diamond-Open-Ring-(1/4-ct.-tw.)-Gold-BE2DP130</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Imogen Pear Diamond Open Ring (1/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/8F/BE2DP130_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/54/BE2DP130_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/51/BE2DP130_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>/Sia-Half-Coverage-Diamond-Ring-(1/8-ct.-tw.)-Gold-BE2D2118P</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Sia Half Coverage Diamond Ring (1/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/37/BE2D2118P_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/1C/BE2D2118P_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/J2/BE2D2118P-yellow_4.jpg, https://image.brilliantearth.com/media/product_new_images/C9/BE2D2118P_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE2D2118P_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/9ff5ff7f-2984-4326-bb9a-d65577132f55</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>/Versailles-Three-Quarter-Coverage-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D621</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Versailles Three-Quarter Coverage Diamond Ring (1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/BA/BE2D621_white_top.jpg, https://image.brilliantearth.com/media/product_images/QM/BE2D621-18KW_4.jpg, https://image.brilliantearth.com/media/product_images/5M/BE2D621-18KW_2.jpg, https://image.brilliantearth.com/media/product_new_images/08/BE2D621_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/26/BE2D621_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/27582cde-1f57-4e2b-9dba-6c00175f11f3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>/Whisper-Half-Coverage-Diamond-Ring-(1/10-ct.-tw.)-White-Gold-BE266</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Whisper Half Coverage Diamond Ring (1/10 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/01/BE266_white_top.jpg, https://image.brilliantearth.com/media/product_images/2X/BE266-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FS/BE4D305-S_BE1D166-18KW_BE266-18KW_2.jpg, https://image.brilliantearth.com/media/product_new_images/C4/BE266_white_side1.jpg, https://image.brilliantearth.com/media/product_images/69/BE266_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/26/BE266_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/0725eb2f-62c0-4ad5-be0b-f711fb129cf9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>/Luxe-Lunette-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D6532</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Luxe Lunette Diamond Ring (1/3 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D6532_white_top.jpg, https://image.brilliantearth.com/media/product_images/NQ/BE2D6532LC-18KW_009.jpg, https://image.brilliantearth.com/media/product_new_images/4E/BE2D6532_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E1/BE2D6532_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/172b3314-e2bb-48e0-b729-47f9ea3c8f93</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>/Ellora-Eternity-Lab-Diamond-Ring-(1-3/4-ct.-tw.)-White-Gold-BE2D2811ETLC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ellora Eternity Lab Diamond Ring (1 3/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/55/BE2D2811ETLC_white_top.jpg, https://image.brilliantearth.com/media/product_images/CM/BE2M2811ET_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/BT/BE2M2811ET_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3E/BE2D2811ETLC_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/be7c5a2a-01e9-43b8-8c71-4697144ede03</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>/Riviera-Eternity-Diamond-Ring-(1-ct.-tw.)-Gold-BE2DR100E</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Riviera Eternity Diamond Ring (1 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/DD/BE2DR100ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR100ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2DR100ELC_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>/Endeavor-7.5mm-Wedding-Ring-Rose-Gold-BE29275</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Endeavor 7.5mm Wedding Ring</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/98/BE29275_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/6B/BE29275_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5A/BE29275_rose_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>/Ellora-Three-Quarter-Coverage-Diamond-Ring-(1-2/5-ct.-tw.)-White-Gold-BE2D8721P</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ellora Three-Quarter Coverage Diamond Ring (1 2/5 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/30/BE2D8721P_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/7A/BE2D8721P_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/0M/BE2D8721P_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/92/BE2D8721P_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BB/BE2D8721P_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>/3mm-Comfort-Fit-Wedding-Ring-Gold-BE207</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3mm Comfort Fit Wedding Ring</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/87/BE207_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/47/BE207_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/KD/BE207-18KY_021.jpg, https://image.brilliantearth.com/media/product_new_images/EE/BE207_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/PB/BE207_yellow_additional1.webp, https://image.brilliantearth.com/media/product_new_images/80/BE207_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>/Olivetta-Half-Coverage-Diamond-Ring-Gold-BE2D15103</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Olivetta Half Coverage Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/2O/BE2D15103_yellow_top_5.jpg, https://image.brilliantearth.com/media/product_new_images/E2/BE2D15103_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/91/BE2D15103_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/FB/BE2D15103_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/7ac48540-8d26-4803-9749-f4bc3815122b</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>/Ulla-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D1136LC</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Ulla Eternity Lab Diamond Ring (1 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/49/BE2D1136LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/A8/BE2D1136LC_rose_additional.jpg, https://image.brilliantearth.com/media/product_new_images/25/BE2D1136LC_rose_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>/Amelie-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2M1056</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Amelie Diamond Ring (1/3 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/06/BE2M1056_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/44/BE2M1056_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VI/BE2M1056_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/28/BE2M1056_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/59/BE2M1056_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/8139940a-4673-45a1-90db-02989682cef9</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>/Petite-Shared-Prong-Three-Quarter-Coverage-Lab-Diamond-Ring-(3/8-ct.-tw.)-White-Gold-BE2PD28R15LC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Petite Shared Prong Three-Quarter Coverage Lab Diamond Ring (3/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/3D/BE2PD28R15_white_top.jpg, https://image.brilliantearth.com/media/product_images/UH/BE2PD28R15-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FI/BE2PD28R15_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/4D/BE2PD28R15_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/65/BE2PD28R15_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>/Bliss-Diamond-Ring-(1/5-ct.-tw.)-White-Gold-BE2FPD14</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bliss Diamond Ring (1/5 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/39/BE2FPD14_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/85/BE2FPD14_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/GO/BE2FPD14-18KW_v2_3.jpg, https://image.brilliantearth.com/media/product_new_images/BE/BE2FPD14_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/82/BE2FPD14_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/55eadf80-4321-4608-b578-3cea16946e51</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>/1.5mm-Quattro-Wedding-Ring-Gold-BE22215</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1.5mm Quattro Wedding Ring</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/60/BE22215_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/FB/BE22215_yellow_hand_lp.jpg, https://image.brilliantearth.com/media/product_images/T5/BE22215_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/DC/BE22215_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/48/BE22215_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/12457e95-7af7-422e-becd-262dd632e937</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>/Sienna-Eternity-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M3420ET</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sienna Eternity Diamond Ring (7/8 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/70/BE2M3420ET_white_top.jpg, https://image.brilliantearth.com/media/product_images/VA/BE2M3420ET-18KW-S6_040.jpg, https://image.brilliantearth.com/media/product_images/KP/BE2M3420-BE2M3420ET-BE2M3420H.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2M3420ET_white_side1.jpg, https://image.brilliantearth.com/media/product_images/DQ/BE2M3420ET_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/18/BE2M3420ET_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>/Wren-Diamond-Open-Ring-White-Gold-BE2D2006</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Wren Diamond Open Ring</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/E3/BE2D2006_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/91/BE2D2006_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/LE/BE2D2006_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/3F/BE2D2006_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B2/BE2D2006_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>/Elongated-Flair-Diamond-Ring-White-Gold-BE2320</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Elongated Flair Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/C8/BE2320_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/49/BE2320_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/C1/BE487343-14KW_053.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2320_white_side1.jpg, https://image.brilliantearth.com/media/product_images/HS/BE2320_white_top_upward.jpg, https://image.brilliantearth.com/media/product_new_images/E5/BE2320_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>/Three-Row-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-White-Gold-BE2D360LC</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Three Row Lab Diamond Ring (1 1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/0F/BE2D360LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/6B/BE2D360LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2D360LC_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>/Sia-Three-Quarter-Coverage-Diamond-Ring-(1/5-ct.-tw.)-White-Gold-BE2D756P</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Sia Three-Quarter Coverage Diamond Ring (1/5 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_images/0R/BE2D756P_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/25/BE2D756P_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/PU/BE2D756P_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/98/BE2D756P_white_side1.jpg, https://image.brilliantearth.com/media/product_images/4S/BE2D756P_white_hand_zi.png</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>/Riviera-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2DR100ELC</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Riviera Eternity Lab Diamond Ring (1 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/DD/BE2DR100ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR100ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2DR100ELC_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>/Astra-Diamond-Ring-Gold-BE2D1112</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Astra Diamond Ring</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/7D/BE2D1112_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/81/BE2D1112_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/PW/BE304RD75-18KY_2.jpg, https://image.brilliantearth.com/media/product_new_images/0A/BE2D1112_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/E9/BE2D1112_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/B5/BE2D1112_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>/Sienna-Half-Coverage-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2M3420H</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sienna Half Coverage Diamond Ring (1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/B2/BE2M3420H_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/AE/BE2M3420H_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/46/BE2M3420H_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/D3/BE2M3420H_white_side1.jpg, https://image.brilliantearth.com/media/product_images/QH/BE2M3420-BE2M3420ET-BE2M3420H.jpeg, https://image.brilliantearth.com/media/product_new_images/AF/BE2M3420H_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>/Petite-Curved-Diamond-Ring-(1/10-ct.-tw.)-White-Gold-BE2D936</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Petite Curved Diamond Ring (1/10 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/99/BE2D936_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/F4/BE2D936_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/UJ/BE2D936-18KW_1.jpg, https://image.brilliantearth.com/media/product_new_images/11/BE2D936_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/52/BE2D936_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/4112bfae-02e1-4285-b960-0553f643cec1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>/Sienna-Three-Quarter-Coverage-Diamond-Open-Ring-(1/2-ct.-tw.)-Gold-BE2D1398</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Sienna Three-Quarter Coverage Diamond Open Ring (1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/B4/BE2D1398_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/XH/BE2D1398-18KW_020.jpg, https://image.brilliantearth.com/media/product_new_images/23/BE2D1398_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D1398_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/7272f794-b967-478e-9f35-fc9ac3cf1e18</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>/Marseille-Three-Quarter-Coverage-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D2774</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Marseille Three-Quarter Coverage Diamond Ring (1/2 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/0B/BE2D2774_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/C1/BE2D2774_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/LM/BE2D2774-yellow.jpg, https://image.brilliantearth.com/media/product_images/YF/BE2D2774_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/9F/BE2D2774_yellow_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>/Versailles-Eternity-Diamond-Ring-(3/4-ct.-tw.)-White-Gold-BE2D1792</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Versailles Eternity Diamond Ring (3/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/F9/BE2D1792_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/A2/BE2D1792_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/CR/850_x_850_BE2D1792_18KW_WG_Eternity_Versailles_WB_product.webp, https://image.brilliantearth.com/media/product_new_images/04/BE2D1792_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A4/BE2D1792_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/c50b4609-4a33-4b1d-88e2-96d7285866a1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>/Delicate-Versailles-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE2D51563</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Delicate Versailles Diamond Ring (1/4 ct. tw.)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D51563_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/16/BE2D51563_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/ED/BE2D51563_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5E/BE2D51563_white_ms_zi.png</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>blob:https://www.brilliantearth.com/24c91c07-70cd-4dfc-b244-291a8b2a6056</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
- Add new scraping files
</commit_message>
<xml_diff>
--- a/brilliantearth_rings/product_data.xlsx
+++ b/brilliantearth_rings/product_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,1004 +446,3109 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Video Link</t>
+          <t>Iframe Link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>/Ballad-Half-Coverage-Diamond-Ring-(1/6-ct.-tw.)-White-Gold-BE2D1823</t>
+          <t>https://www.brilliantearth.com/Adorned-Petite-Twisted-Vine-Three-Stone-Diamond-Ring-Rose-Gold-BE1D3043-25508894/</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ballad Half Coverage Diamond Ring (1/6 ct. tw.)</t>
+          <t>Adorned Petite Twisted Vine Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/5F/BE2D1823_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/8B/BE2D1823_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/BN/BE2D1823E_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/75/BE2D1823_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/2A/BE2D1823_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/4P/BE1D3043_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/EF/BE1D3043_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/FF/BE1D3043_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/5L/BE1D3043_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/560288768?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>/Nouveau-Diamond-Ring-White-Gold-BE2D2359</t>
+          <t>https://www.brilliantearth.com/Briar-Diamond-Ring-Rose-Gold-BE1D25344-19515933/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nouveau Diamond Ring</t>
+          <t>Briar Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/D8/BE2D2359_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/5F/BE2D2359_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/20/BE2D2359_white_additional1.jpeg, https://image.brilliantearth.com/media/product_images/71/BE2D2359_white_02.jpg, https://image.brilliantearth.com/media/product_images/T8/BE2D2359_white_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/4W/BE1D25344_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/56/BE1D25344_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/2D/BE1D25344_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/59/BE1D25344_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/FA/BE1D25344_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/9280ce70-8718-4319-9e49-abecb31c67c1</t>
+          <t>embed.imajize.com/6452249?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>/Matte-Hammered-Petite-Comfort-Fit-Wedding-Ring-Gold-BE299MH</t>
+          <t>https://www.brilliantearth.com/Aimee-Open-Double-Band-Solitaire-Ring-Rose-Gold-BE14122-20969829/</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Matte Hammered Petite Comfort Fit Wedding Ring</t>
+          <t>Aimee Open Double Band Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/J0/BE299MH_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE299MH_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/DT/BE299MH_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_images/ER/BE299MH_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/3C/BE299MH_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/FB/BE14122_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/B5/BE14122_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/6F/BE14122_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/AJ/BE14122_rose_Emerald_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/0b514589-c8b9-425f-9f18-c34f895c60bf</t>
+          <t>embed.imajize.com/2318645?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>/Jardiniere-Diamond-Ring-Gold-BE2D835</t>
+          <t>https://www.brilliantearth.com/Petite-Cometa-Perfect-Fit-Three-Stone-Diamond-Ring-Rose-Gold-BE1D5400-17095659/</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jardiniere Diamond Ring</t>
+          <t>Petite Cometa Perfect Fit Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/CD/BE2D835_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/PJ/BE2D835-18KY_2.jpg, https://image.brilliantearth.com/media/product_images/76/BE2D835-18KY_3.jpg, https://image.brilliantearth.com/media/product_new_images/52/BE2D835_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/48/BE2D835_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/E5/BE2D835_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/S8/BE1D5400_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/30/BE1D5400_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/87/BE1D5400_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B1/BE1D5400_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/MY/BE1D5400_rose_Marquise_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/78d6962e-0b2f-418b-9d24-ea42837fdf1e</t>
+          <t>embed.imajize.com/485461519?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>/Luxe-Winding-Willow-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE2564LD</t>
+          <t>https://www.brilliantearth.com/Adorned-Amelie-Diamond-Ring-Rose-Gold-BE1D1467-22120996/</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Luxe Winding Willow Diamond Ring (1/4 ct. tw.)</t>
+          <t>Adorned Amelie Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/90/BE2564LD_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/04/BE2564LD_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/E4/BE2564LD-18KW.jpg, https://image.brilliantearth.com/media/product_images/3H/BE2564LD_white_side.jpg, https://image.brilliantearth.com/media/product_images/42/BE2564LD_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/92/BE2564LD_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/RS/BE1D1467_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/64/BE1D1467_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F7/BE1D1467_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/XI/BE1D1467_rose_Round_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/8fd59de9-323f-46d6-820b-fcef0eeb7748</t>
+          <t>embed.imajize.com/746413729?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>/Petite-Shared-Prong-Three-Quarter-Coverage-Diamond-Ring-(3/8-ct.-tw.)-White-Gold-BE2PD28R15</t>
+          <t>https://www.brilliantearth.com/Camellia-Three-Stone-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D2470-17410552/</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Petite Shared Prong Three-Quarter Coverage Diamond Ring (3/8 ct. tw.)</t>
+          <t>Camellia Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/3D/BE2PD28R15_white_top.jpg, https://image.brilliantearth.com/media/product_images/UH/BE2PD28R15-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FI/BE2PD28R15_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/4D/BE2PD28R15_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/65/BE2PD28R15_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/OZ/BE1D2470_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/A3/BE1D2470_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/D7/BE1D2470_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E8/BE1D2470_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/4E/BE1D2470_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/60cab62e-85bb-4423-8f3f-9a7b5126fccb</t>
+          <t>embed.imajize.com/8252076?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>/Riviera-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Gold-BE2DR200ELC</t>
+          <t>https://www.brilliantearth.com/Petite-Secret-Halo-Diamond-Ring-Rose-Gold-BE1D3108-17281915/</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Riviera Eternity Lab Diamond Ring (2 ct. tw.)</t>
+          <t>Petite Secret Halo Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/D1/BE2DR200ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/A8/BE2DR200ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A7/BE2DR200ELC_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/KN/BE1D3108_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/60/BE1D3108_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/68/BE1D3108_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/33/BE1D3108_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/GN/BE1D3108_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/545235998?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>/Versailles-Eternity-Lab-Diamond-Ring-(3/4-ct.-tw.)-Gold-BE2D1792LC</t>
+          <t>https://www.brilliantearth.com/Waverly-Halo-Diamond-Ring-with-Black-Diamond-Accents-Rose-Gold-BE1D3244-12776471/</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Versailles Eternity Lab Diamond Ring (3/4 ct. tw.)</t>
+          <t>Waverly Halo Diamond Engagement Ring with Black Diamond Accents</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/96/BE2D1792_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/NE/BE2D1792-yellow_019.jpg, https://image.brilliantearth.com/media/product_new_images/E6/BE2D1792_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/64/BE2D1792_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/W2/BE1D3244_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/19/BE1D3244_PS_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/CA/BE1D3244_PS_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/DZ/BE1D3244_rose_Pear_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/87e958c6-e357-430a-a2ea-581c5c3ebf07</t>
+          <t>embed.imajize.com/3419734?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>/Sienna-Eternity-Lab-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M3420ETLC</t>
+          <t>https://www.brilliantearth.com/Adorned-Tapered-Baguette-Three-Stone-Diamond-Ring-Rose-Gold-BE1D5507-19670916/</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sienna Eternity Lab Diamond Ring (7/8 ct. tw.)</t>
+          <t>Adorned Tapered Baguette Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/70/BE2M3420ET_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2M3420ETLC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/KP/BE2M3420-BE2M3420ET-BE2M3420H.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2M3420ET_white_side1.jpg, https://image.brilliantearth.com/media/product_images/DQ/BE2M3420ET_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/18/BE2M3420ET_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/YT/BE1D5507_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/4E/BE1D5507_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/80/BE1D5507_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/PM/BE1D5507_rose_Emerald_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/2a84a988-a1cc-43f8-bb15-4ed049e33998</t>
+          <t>embed.imajize.com/4937512?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>/Luxe-Tiara-Eternity-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D147E</t>
+          <t>https://www.brilliantearth.com/Lotus-Flower-Halo-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE1BD12R2-1152409/</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18K White Gold
-            Luxe Tiara Eternity Diamond Ring (1/2 ct. tw.)</t>
+          <t>Lotus Flower Halo Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/A8/BE2D147E_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/AA/BE2D147E_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/7L/BE2D147E_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/DA/BE2D147E_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/6C/BE2D147E_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/RH/BE1BD12R2_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/8E/BE1BD12R2_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/K6/BE1BD12R2_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/0B/BE1BD12R2_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B1/BE1BD12R2_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/XB/BE1BD12R2_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/4819583?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>/Riviera-Eternity-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2DR200E</t>
+          <t>https://www.brilliantearth.com/Camellia-Three-Stone-Pear-Diamond-Ring-Rose-Gold-BE1D2486-23803863/</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Riviera Eternity Diamond Ring (2 ct. tw.)</t>
+          <t>Camellia Three Stone Pear Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/9A/BE2DR200ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/9F/BE2DR200ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/78/BE2DR200ELC_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/YA/BE1D2486_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_images/PL/BE1D2486_rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/20/BE1D2486_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/60/BE1D2486_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/AD/BE1D2486_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/157183894?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>/Whisper-Eternity-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE266E</t>
+          <t>https://www.brilliantearth.com/Trillion-Cut-Three-Stone-Diamond-Ring-Rose-Gold-BE1D233-1964872/</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Whisper Eternity Diamond Ring (1/4 ct. tw.)</t>
+          <t>Trillion Cut Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/8C/BE266E_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/80/BE266E_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/FW/BE266E_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/84/BE266E_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/88/BE266E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/EM/BE1D233_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/1D/BE1D233_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/6T/BE1D233_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/97/BE1D233_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/37/BE1D233_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/9Z/BE1D233_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/f47739af-c394-4d3d-9c27-88895be403d6</t>
+          <t>embed.imajize.com/924219308?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>/Flair-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D1938</t>
+          <t>https://www.brilliantearth.com/Chamise-Hidden-Halo-Diamond-Ring-Rose-Gold-BE1D288-23748041/</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Flair Diamond Ring (1/3 ct. tw.)</t>
+          <t>Chamise Hidden Halo Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/85/BE2D1938_white_top.jpg, https://image.brilliantearth.com/media/product_images/2V/BE2D1938.jpeg, https://image.brilliantearth.com/media/product_images/NW/BE2D1938_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/00/BE2D1938_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D7/BE2D1938_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/JS/BE1D288_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/F3/BE1D288_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/8A/BE1D288_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/K0/BE1D288_rose_Round_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/32238343-5dbf-4d21-a6f9-0dadece8c4ff</t>
+          <t>embed.imajize.com/722917948?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>/Monaco-Diamond-Ring-(3/4-ct.-tw.)-White-Gold-BE2D829</t>
+          <t>https://www.brilliantearth.com/Luna-Hidden-Halo-Diamond-Ring-Rose-Gold-BE1D1678-23785358/</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Monaco Diamond Ring (3/4 ct. tw.)</t>
+          <t>Luna Hidden Halo Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/35/BE2D829_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/D3/BE2D829_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/W2/BE2D829_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/CC/BE2D829_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/DC/BE2D829_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/H7/BE1D1678_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_images/FX/BE1D1678_rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/55/BE1D1678_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/42/BE1D1678_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/LD/BE1D1678_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/753632610?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>/Ellora-Half-Coverage-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M2811</t>
+          <t>https://www.brilliantearth.com/Tabitha-Channel-Set-Baguette-Diamond-Ring-Rose-Gold-BE1D118-27546203/</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ellora Half Coverage Diamond Ring (7/8 ct. tw.)</t>
+          <t>Tabitha Channel Set Baguette Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/06/BE2M2811_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/0D/BE2M2811_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/D2/BE2M2811_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/8D/BE2M2811_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/H3/BE1D118_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/39/BE1D118_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/28/BE1D118_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/NV/BE1D118_rose_Round_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/d4489832-4a72-41f8-892c-e0f44d0d3ec1</t>
+          <t>embed.imajize.com/922667909?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>/Curved-Versailles-Diamond-Ring-White-Gold-BE2D7422</t>
+          <t>https://www.brilliantearth.com/Amelie-Three-Quarter-Coverage-Diamond-Ring-Rose-Gold-BE1D7162-14690551/</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Curved Versailles Diamond Ring</t>
+          <t>Amelie Three-Quarter Coverage Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AC/BE2D7422_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/02/BE2D7422_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VK/BE2D7422_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Z5/BE1D7162_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/44/BE1D7162_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E6/BE1D7162_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/AW/BE1D7162_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/239331219?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>/Entwined-Diamond-Contour-Ring-(1/5-ct.-tw.)-Rose-Gold-BE2D1816</t>
+          <t>https://www.brilliantearth.com/Luxe-Three-Stone-Petite-Twisted-Vine-Diamond-Ring-Rose-Gold-BE1D3055-16829087/</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Entwined Diamond Contour Ring (1/5 ct. tw.)</t>
+          <t>Luxe Three Stone Petite Twisted Vine Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/B3/BE2D1816_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/35/BE2D1816_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E7/BE2D1816_rose_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/IL/BE1D3055_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/84/BE1D3055_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/DE/BE1D3055_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/12/BE1D3055_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/ZN/BE1D3055_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/1976574?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>/Sia-Half-Coverage-Lab-Diamond-Ring-(1/8-ct.-tw.)-Gold-BE2D2118PLC</t>
+          <t>https://www.brilliantearth.com/Valencia-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D3907-26361706/</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sia Half Coverage Lab Diamond Ring (1/8 ct. tw.)</t>
+          <t>Valencia Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/37/BE2D2118P_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/9C/BE2D2118P-yellow_2.jpg, https://image.brilliantearth.com/media/product_images/J2/BE2D2118P-yellow_4.jpg, https://image.brilliantearth.com/media/product_new_images/C9/BE2D2118P_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE2D2118P_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/RK/BE1D3907_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/4X/BE1D3907_rose_harmony1.jpg, https://image.brilliantearth.com/media/product_images/Y2/BE1D3907_rose_harmony2.jpg, https://image.brilliantearth.com/media/carat_image/57/BE1D3907_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/46/BE1D3907_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/product_images/X4/BE1D3907_rose_harmony3.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/OL/BE1D3907_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/598834548?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>/Chevron-Ring-Gold-BE2119</t>
+          <t>https://www.brilliantearth.com/Yvonne-Diamond-Ring-Rose-Gold-BE1D3066-18560855/</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Chevron Ring</t>
+          <t>Yvonne Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/55/BE2119_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/50/BE2119_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/U6/YG2.jpg, https://image.brilliantearth.com/media/product_new_images/D0/BE2119_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/TJ/BE1D3066_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/51/BE1D3066_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/E9/BE1D3066_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/AE/BE1D3066_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/4P/BE1D3066_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/26bc93b2-094f-4a94-98f3-c942a4ef09eb</t>
+          <t>embed.imajize.com/471947803?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>/Curved-Versailles-Lab-Diamond-Ring-White-Gold-BE2D7422LC</t>
+          <t>https://www.brilliantearth.com/Zinnia-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D1610-2268399/</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Curved Versailles Lab Diamond Ring</t>
+          <t>Zinnia Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AC/BE2D7422_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/02/BE2D7422_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VK/BE2D7422_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/XH/BE1D1610_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/8F/BE1D1610_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/KM/BE1D1610_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/89/BE1D1610_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B8/BE1D1610_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/1B/BE1D1610_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/843887989?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>/Gemma-Baguette-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D084B</t>
+          <t>https://www.brilliantearth.com/Noemi-Bezel-Ring-Rose-Gold-BE1808-11522153/</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Gemma Baguette Diamond Ring (1/2 ct. tw.)</t>
+          <t>Noemi Bezel Engagement Ring</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/A6/BE2D084B_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/5A/BE2D084B_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/3F/BE2D084B_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/7R/BE2D084B_yellow_side.jpeg, https://image.brilliantearth.com/media/product_new_images/FD/BE2D084B_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/0F/BE1808_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/6C/BE1808_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/47/BE1808_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/D3/BE1808_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/669743054?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>/Imogen-Pear-Diamond-Open-Ring-(1/4-ct.-tw.)-Gold-BE2DP130</t>
+          <t>https://www.brilliantearth.com/Nadia-Sapphire-and-Diamond-Ring-Rose-Gold-BE1S6013-21490784/</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Imogen Pear Diamond Open Ring (1/4 ct. tw.)</t>
+          <t>Nadia Sapphire and Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/8F/BE2DP130_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/54/BE2DP130_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/51/BE2DP130_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/2N/BE1S6013_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/BE/BE1S6013_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/1D/BE1S6013_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/SK/BE1S6013_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/6949704?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>/Sia-Half-Coverage-Diamond-Ring-(1/8-ct.-tw.)-Gold-BE2D2118P</t>
+          <t>https://www.brilliantearth.com/Hudson-Engraved-Diamond-Ring-Rose-Gold-BE132D-3940072/</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sia Half Coverage Diamond Ring (1/8 ct. tw.)</t>
+          <t>Hudson Engraved Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/37/BE2D2118P_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/1C/BE2D2118P_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/J2/BE2D2118P-yellow_4.jpg, https://image.brilliantearth.com/media/product_new_images/C9/BE2D2118P_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE2D2118P_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/OQ/BE132D_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/AF/BE132D_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/C8/BE132D_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/CA/BE132D_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/F8/BE132D_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/9ff5ff7f-2984-4326-bb9a-d65577132f55</t>
+          <t>embed.imajize.com/859490674?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>/Versailles-Three-Quarter-Coverage-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D621</t>
+          <t>https://www.brilliantearth.com/East-West-Tapered-Baguette-Diamond-Ring-Rose-Gold-BE1D1964-16189742/</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Versailles Three-Quarter Coverage Diamond Ring (1/2 ct. tw.)</t>
+          <t>East West Tapered Baguette Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/BA/BE2D621_white_top.jpg, https://image.brilliantearth.com/media/product_images/QM/BE2D621-18KW_4.jpg, https://image.brilliantearth.com/media/product_images/5M/BE2D621-18KW_2.jpg, https://image.brilliantearth.com/media/product_new_images/08/BE2D621_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/26/BE2D621_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/base_product_center_diamond_images/HI/BE1D1964_HorizontalBead_Emerald_rose_carat_125.jpg, https://image.brilliantearth.com/media/product_images/N8/BE082_BE1D1964LC-rose_006.jpg, https://image.brilliantearth.com/media/product_images/DU/BE1D1964_rose_side.jpg, https://image.brilliantearth.com/media/base_product_center_diamond_images/H2/BE1D1964_HorizontalBead_Emerald_rose_carat_125_hd_zo.png</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/27582cde-1f57-4e2b-9dba-6c00175f11f3</t>
+          <t>embed.imajize.com/210402153?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>/Whisper-Half-Coverage-Diamond-Ring-(1/10-ct.-tw.)-White-Gold-BE266</t>
+          <t>https://www.brilliantearth.com/Adorned-Luxe-Petite-Twisted-Vine-Diamond-Ring-Rose-Gold-BE1D1432-22323656/</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Whisper Half Coverage Diamond Ring (1/10 ct. tw.)</t>
+          <t>Adorned Luxe Petite Twisted Vine Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/01/BE266_white_top.jpg, https://image.brilliantearth.com/media/product_images/2X/BE266-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FS/BE4D305-S_BE1D166-18KW_BE266-18KW_2.jpg, https://image.brilliantearth.com/media/product_new_images/C4/BE266_white_side1.jpg, https://image.brilliantearth.com/media/product_images/69/BE266_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/26/BE266_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/DT/BE1D1432_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/C7/BE1D1432_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2A/BE1D1432_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/8U/BE1D1432_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/0725eb2f-62c0-4ad5-be0b-f711fb129cf9</t>
+          <t>embed.imajize.com/727099679?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>/Luxe-Lunette-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D6532</t>
+          <t>https://www.brilliantearth.com/Delicate-Shared-Prong-Diamond-Ring-Rose-Gold-BE1D6060-17418277/</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Luxe Lunette Diamond Ring (1/3 ct. tw.)</t>
+          <t>Delicate Shared Prong Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D6532_white_top.jpg, https://image.brilliantearth.com/media/product_images/NQ/BE2D6532LC-18KW_009.jpg, https://image.brilliantearth.com/media/product_new_images/4E/BE2D6532_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E1/BE2D6532_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/42/BE1D6060_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/B5/BE1D6060_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B9/BE1D6060_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/VG/BE1D6060_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/172b3314-e2bb-48e0-b729-47f9ea3c8f93</t>
+          <t>embed.imajize.com/7927867?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>/Ellora-Eternity-Lab-Diamond-Ring-(1-3/4-ct.-tw.)-White-Gold-BE2D2811ETLC</t>
+          <t>https://www.brilliantearth.com/Sweeping-Ivy-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D4513-8724788/</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ellora Eternity Lab Diamond Ring (1 3/4 ct. tw.)</t>
+          <t>Sweeping Ivy Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/55/BE2D2811ETLC_white_top.jpg, https://image.brilliantearth.com/media/product_images/CM/BE2M2811ET_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/BT/BE2M2811ET_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3E/BE2D2811ETLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/base_product_center_diamond_images/JP/BE1D4513_sweepingvine_Pear_rose_carat_2.jpg, https://image.brilliantearth.com/media/product_images/AK/BE1D4513-BE2D5422_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/AF/BE1D4513_rose_side.jpg, https://image.brilliantearth.com/media/base_product_center_diamond_images/U7/BE1D4513_sweepingvine_Pear_rose_carat_2_hd_zo.png</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/be7c5a2a-01e9-43b8-8c71-4697144ede03</t>
+          <t>embed.imajize.com/9098675?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>/Riviera-Eternity-Diamond-Ring-(1-ct.-tw.)-Gold-BE2DR100E</t>
+          <t>https://www.brilliantearth.com/Monsella-Solitaire-Ring-Rose-Gold-BE1484-12694818/</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Riviera Eternity Diamond Ring (1 ct. tw.)</t>
+          <t>Monsella Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/DD/BE2DR100ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR100ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2DR100ELC_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/XB/BE1484_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/product_images/0K/BE1484-rose_060.jpg, https://image.brilliantearth.com/media/carat_image/3D/BE1484_PS_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/0A/BE1484_PS_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/WY/BE1484_rose_Pear_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/4982630?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>/Endeavor-7.5mm-Wedding-Ring-Rose-Gold-BE29275</t>
+          <t>https://www.brilliantearth.com/Summer-Blossom-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE1D9683-8724778/</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Endeavor 7.5mm Wedding Ring</t>
+          <t>Summer Blossom Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/98/BE29275_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/6B/BE29275_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5A/BE29275_rose_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/3N/BE1D9683_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/89/BE1D9683_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/4B/BE1D9683_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F7/BE1D9683_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/PS/BE1D9683_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/651593145?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>/Ellora-Three-Quarter-Coverage-Diamond-Ring-(1-2/5-ct.-tw.)-White-Gold-BE2D8721P</t>
+          <t>https://www.brilliantearth.com/Ballad-Three-Quarter-Coverage-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE164-3015402/</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ellora Three-Quarter Coverage Diamond Ring (1 2/5 ct. tw.)</t>
+          <t>Ballad Three-Quarter Coverage Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/30/BE2D8721P_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/7A/BE2D8721P_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/0M/BE2D8721P_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/92/BE2D8721P_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BB/BE2D8721P_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/QG/BE164_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/1A/BE164_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/5B/BE164_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/6B/BE164_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B0/BE164_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/JE/BE164_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/830792853?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>/3mm-Comfort-Fit-Wedding-Ring-Gold-BE207</t>
+          <t>https://www.brilliantearth.com/Celestia-Milgrain-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE1D8102-19452836/</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>3mm Comfort Fit Wedding Ring</t>
+          <t>Celestia Milgrain Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/87/BE207_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/47/BE207_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/KD/BE207-18KY_021.jpg, https://image.brilliantearth.com/media/product_new_images/EE/BE207_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/PB/BE207_yellow_additional1.webp, https://image.brilliantearth.com/media/product_new_images/80/BE207_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/E6/BE1D8102_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/77/BE1D8102_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/74/BE1D8102_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/EA/BE1D8102_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/805222257?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>/Olivetta-Half-Coverage-Diamond-Ring-Gold-BE2D15103</t>
+          <t>https://www.brilliantearth.com/Waverly-Hidden-Halo-Diamond-Ring-Rose-Gold-BE1D9392-19452780/</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Olivetta Half Coverage Diamond Ring</t>
+          <t>Waverly Hidden Halo Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/2O/BE2D15103_yellow_top_5.jpg, https://image.brilliantearth.com/media/product_new_images/E2/BE2D15103_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/91/BE2D15103_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/FB/BE2D15103_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/G4/BE1D9392_rose_Cushion_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/46/BE1D9392_CU_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2E/BE1D9392_CU_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/D3/BE1D9392_rose_Cushion_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/7ac48540-8d26-4803-9749-f4bc3815122b</t>
+          <t>embed.imajize.com/802274968?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>/Ulla-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D1136LC</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Ulla Eternity Lab Diamond Ring (1 ct. tw.)</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/49/BE2D1136LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/A8/BE2D1136LC_rose_additional.jpg, https://image.brilliantearth.com/media/product_new_images/25/BE2D1136LC_rose_ms_zi.png</t>
-        </is>
-      </c>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Classic-Diamond-Ring-(1/5-ct.-tw.)-Rose-Gold-BE1DT2670-10982702/</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>/Amelie-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2M1056</t>
+          <t>https://www.brilliantearth.com/Hazel-Solitaire-Ring-Rose-Gold-BE1983-4554010/</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Amelie Diamond Ring (1/3 ct. tw.)</t>
+          <t>Hazel Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/06/BE2M1056_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/44/BE2M1056_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VI/BE2M1056_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/28/BE2M1056_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/59/BE2M1056_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/DU/BE1983_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/9F/BE1983_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/LP/BE1983_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/32/BE1983_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/63/BE1983_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/WZ/BE1983_rose_Emerald_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/8139940a-4673-45a1-90db-02989682cef9</t>
+          <t>embed.imajize.com/3943575?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>/Petite-Shared-Prong-Three-Quarter-Coverage-Lab-Diamond-Ring-(3/8-ct.-tw.)-White-Gold-BE2PD28R15LC</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Petite Shared Prong Three-Quarter Coverage Lab Diamond Ring (3/8 ct. tw.)</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/3D/BE2PD28R15_white_top.jpg, https://image.brilliantearth.com/media/product_images/UH/BE2PD28R15-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FI/BE2PD28R15_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/4D/BE2PD28R15_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/65/BE2PD28R15_white_ms_zi.png</t>
-        </is>
-      </c>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Cathedral-Drape-Diamond-Ring-Rose-Gold-BE1DT2684-12921122/</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>/Bliss-Diamond-Ring-(1/5-ct.-tw.)-White-Gold-BE2FPD14</t>
+          <t>https://www.brilliantearth.com/Perfect-Fit-Tapered-Baguette-Diamond-Ring-Rose-Gold-BE1D454-27546198/</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bliss Diamond Ring (1/5 ct. tw.)</t>
+          <t>Perfect Fit Tapered Baguette Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/39/BE2FPD14_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/85/BE2FPD14_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/GO/BE2FPD14-18KW_v2_3.jpg, https://image.brilliantearth.com/media/product_new_images/BE/BE2FPD14_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/82/BE2FPD14_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/EM/BE1D454_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/4B/BE1D454_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/1D/BE1D454_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/BW/BE1D454_rose_Emerald_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/55eadf80-4321-4608-b578-3cea16946e51</t>
+          <t>embed.imajize.com/981008620?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>/1.5mm-Quattro-Wedding-Ring-Gold-BE22215</t>
+          <t>https://www.brilliantearth.com/Twisted-Vine-Hidden-Halo-Diamond-Ring-Rose-Gold-BE1D567-24075679/</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1.5mm Quattro Wedding Ring</t>
+          <t>Twisted Vine Hidden Halo Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/60/BE22215_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/FB/BE22215_yellow_hand_lp.jpg, https://image.brilliantearth.com/media/product_images/T5/BE22215_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/DC/BE22215_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/48/BE22215_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/R5/BE1D567_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/55/BE1D567_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F1/BE1D567_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/R8/BE1D567_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/12457e95-7af7-422e-becd-262dd632e937</t>
+          <t>embed.imajize.com/244608112?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>/Sienna-Eternity-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M3420ET</t>
+          <t>https://www.brilliantearth.com/Luxe-Trillion-Cut-Three-Stone-Diamond-Ring-Rose-Gold-BE1D234-18472814/</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Sienna Eternity Diamond Ring (7/8 ct. tw.)</t>
+          <t>Luxe Trillion Cut Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/70/BE2M3420ET_white_top.jpg, https://image.brilliantearth.com/media/product_images/VA/BE2M3420ET-18KW-S6_040.jpg, https://image.brilliantearth.com/media/product_images/KP/BE2M3420-BE2M3420ET-BE2M3420H.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2M3420ET_white_side1.jpg, https://image.brilliantearth.com/media/product_images/DQ/BE2M3420ET_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/18/BE2M3420ET_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/BD/BE1D234_rose_Cushion_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/5E/BE1D234_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/FC/BE1D234_CU_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/78/BE1D234_CU_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/QK/BE1D234_rose_Cushion_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/2157367?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>/Wren-Diamond-Open-Ring-White-Gold-BE2D2006</t>
+          <t>https://www.brilliantearth.com/Icon-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D005-10595133/</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Wren Diamond Open Ring</t>
+          <t>Icon Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/E3/BE2D2006_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/91/BE2D2006_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/LE/BE2D2006_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/3F/BE2D2006_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B2/BE2D2006_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/3J/BE1D005_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/product_images/Y4/BE1D005_rose_O-PROFILE.jpg, https://image.brilliantearth.com/media/product_images/YX/Icon--Luxe-Heritage-.jpg, https://image.brilliantearth.com/media/carat_image/06/BE1D005_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/89/BE1D005_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/95/BE1D005_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/104503057?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>/Elongated-Flair-Diamond-Ring-White-Gold-BE2320</t>
+          <t>https://www.brilliantearth.com/Alden-Diamond-Ring-Rose-Gold-BE1D303-11196205/</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Elongated Flair Diamond Ring</t>
+          <t>Alden Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/C8/BE2320_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/49/BE2320_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/C1/BE487343-14KW_053.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2320_white_side1.jpg, https://image.brilliantearth.com/media/product_images/HS/BE2320_white_top_upward.jpg, https://image.brilliantearth.com/media/product_new_images/E5/BE2320_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/P3/BE1D303_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/A8/BE1D303_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/29/BE1D303_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/JH/BE1D303_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/197518180?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>/Three-Row-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-White-Gold-BE2D360LC</t>
+          <t>https://www.brilliantearth.com/Camellia-Indigo-Milgrain-Ring-Rose-Gold-BE1D2468AQ-19184644/</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Three Row Lab Diamond Ring (1 1/2 ct. tw.)</t>
+          <t>Camellia Indigo Milgrain Engagement Ring</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/0F/BE2D360LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/6B/BE2D360LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2D360LC_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/7O/BE1D2468AQ_rose_Pear_top_125_carat.png, https://image.brilliantearth.com/media/product_new_images/BC/BE1D2468AQ_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/0E/BE1D2468AQ_PE_125ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/93/BE1D2468AQ_PE_125ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/Y3/BE1D2468AQ_rose_Pear_hand_zo_125_carat.png</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/904308849?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>/Sia-Three-Quarter-Coverage-Diamond-Ring-(1/5-ct.-tw.)-White-Gold-BE2D756P</t>
+          <t>https://www.brilliantearth.com/Perfect-Fit-East-West-Solitaire-Ring-Rose-Gold-BE19880-21809063/</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Sia Three-Quarter Coverage Diamond Ring (1/5 ct. tw.)</t>
+          <t>Perfect Fit East-West Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/0R/BE2D756P_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/25/BE2D756P_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/PU/BE2D756P_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/98/BE2D756P_white_side1.jpg, https://image.brilliantearth.com/media/product_images/4S/BE2D756P_white_hand_zi.png</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/base_product_center_diamond_images/LI/BE19880_horizontalclaw_Emerald_rose_carat_2.jpg, https://image.brilliantearth.com/media/product_images/HP/BE19880_rose_side.jpg, https://image.brilliantearth.com/media/base_product_center_diamond_images/90/BE19880_horizontalclaw_Emerald_rose_carat_2_hd_zo.png</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/715166908?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>/Riviera-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2DR100ELC</t>
+          <t>https://www.brilliantearth.com/Luz-Baguette-and-Round-Diamond-Ring-Rose-Gold-BE1D4477-20319013/</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Riviera Eternity Lab Diamond Ring (1 ct. tw.)</t>
+          <t>Luz Baguette and Round Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/DD/BE2DR100ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR100ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2DR100ELC_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/3S/BE1D4477_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/6E/BE1D4477_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/BD/BE1D4477_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/2W/BE1D4477_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/7892835?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>/Astra-Diamond-Ring-Gold-BE2D1112</t>
+          <t>https://www.brilliantearth.com/Luxe-Cometa-Hidden-Accent-Diamond-Ring-Rose-Gold-BE1D1723-23803868/</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Astra Diamond Ring</t>
+          <t>Luxe Cometa Hidden Accent Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/7D/BE2D1112_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/81/BE2D1112_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/PW/BE304RD75-18KY_2.jpg, https://image.brilliantearth.com/media/product_new_images/0A/BE2D1112_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/E9/BE2D1112_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/B5/BE2D1112_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Z7/BE1D1723_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/product_images/PF/BE1D1723_rose_F_model.JPG, https://image.brilliantearth.com/media/carat_image/D4/BE1D1723_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/35/BE1D1723_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/V0/BE1D1723_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/125798967?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>/Sienna-Half-Coverage-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2M3420H</t>
+          <t>https://www.brilliantearth.com/Whisper-Diamond-Ring-Rose-Gold-BE1D6339-20195176/</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Sienna Half Coverage Diamond Ring (1/2 ct. tw.)</t>
+          <t>Whisper Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/B2/BE2M3420H_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/AE/BE2M3420H_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/46/BE2M3420H_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/D3/BE2M3420H_white_side1.jpg, https://image.brilliantearth.com/media/product_images/QH/BE2M3420-BE2M3420ET-BE2M3420H.jpeg, https://image.brilliantearth.com/media/product_new_images/AF/BE2M3420H_white_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/4A/BE1D6339_rose_Radiant_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/33/BE1D6339_RA_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/31/BE1D6339_RA_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/AN/BE1D6339_rose_Radiant_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/7226623?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>/Petite-Curved-Diamond-Ring-(1/10-ct.-tw.)-White-Gold-BE2D936</t>
+          <t>https://www.brilliantearth.com/Chantal-Diamond-Ring-Rose-Gold-BE1D9213-12694834/</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Petite Curved Diamond Ring (1/10 ct. tw.)</t>
+          <t>Chantal Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/99/BE2D936_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/F4/BE2D936_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/UJ/BE2D936-18KW_1.jpg, https://image.brilliantearth.com/media/product_new_images/11/BE2D936_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/52/BE2D936_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/5W/BE1D9213_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/8A/BE1D9213_PS_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/A4/BE1D9213_PS_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/2O/BE1D9213_rose_Pear_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/4112bfae-02e1-4285-b960-0553f643cec1</t>
+          <t>embed.imajize.com/505386144?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>/Sienna-Three-Quarter-Coverage-Diamond-Open-Ring-(1/2-ct.-tw.)-Gold-BE2D1398</t>
+          <t>https://www.brilliantearth.com/Amaranta-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D1032-13470555/</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Sienna Three-Quarter Coverage Diamond Open Ring (1/2 ct. tw.)</t>
+          <t>Amaranta Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/B4/BE2D1398_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/XH/BE2D1398-18KW_020.jpg, https://image.brilliantearth.com/media/product_new_images/23/BE2D1398_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D1398_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/0H/BE1D1032_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_images/XJ/850x850_03_MAR2022_OF_ER_WildflowerHero_056.jpg, https://image.brilliantearth.com/media/carat_image/80/BE1D1032_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/D5/BE1D1032_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/YP/BE1D1032_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/7272f794-b967-478e-9f35-fc9ac3cf1e18</t>
+          <t>embed.imajize.com/902832115?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>/Marseille-Three-Quarter-Coverage-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D2774</t>
+          <t>https://www.brilliantearth.com/Sienna-Half-Coverage-Hidden-Accents-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D3248-23608722/</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Marseille Three-Quarter Coverage Diamond Ring (1/2 ct. tw.)</t>
+          <t>Sienna Half Coverage Hidden Accents Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/0B/BE2D2774_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/C1/BE2D2774_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/LM/BE2D2774-yellow.jpg, https://image.brilliantearth.com/media/product_images/YF/BE2D2774_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/9F/BE2D2774_yellow_ms_zi.png</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/82/BE1D3248_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/83/BE1D3248_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/3E/BE1D3248_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/5U/BE1D3248_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/373334438?v=1739347866</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>/Versailles-Eternity-Diamond-Ring-(3/4-ct.-tw.)-White-Gold-BE2D1792</t>
+          <t>https://www.brilliantearth.com/Secret-Garden-Gallery-Three-Stone-Diamond-Ring-Rose-Gold-BE1D6563-22635112/</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Versailles Eternity Diamond Ring (3/4 ct. tw.)</t>
+          <t>Secret Garden Gallery Three Stone Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/F9/BE2D1792_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/A2/BE2D1792_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/CR/850_x_850_BE2D1792_18KW_WG_Eternity_Versailles_WB_product.webp, https://image.brilliantearth.com/media/product_new_images/04/BE2D1792_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A4/BE2D1792_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/4K/BE1D6563_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/20/BE1D6563_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/EA/BE1D6563_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/3V/BE1D6563_rose_Oval_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/c50b4609-4a33-4b1d-88e2-96d7285866a1</t>
+          <t>embed.imajize.com/678338885?v=1739347866</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>/Delicate-Versailles-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE2D51563</t>
+          <t>https://www.brilliantearth.com/Sonora-Diamond-Ring-Rose-Gold-BE110-1152696/</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Delicate Versailles Diamond Ring (1/4 ct. tw.)</t>
+          <t>Sonora Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D51563_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/16/BE2D51563_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/ED/BE2D51563_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5E/BE2D51563_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/1S/BE110_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/A1/BE110_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/KL/BE110_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/2B/BE110_PS_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F6/BE110_PS_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/E1/BE110_rose_Pear_hand_zo_2_carat.png</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>blob:https://www.brilliantearth.com/24c91c07-70cd-4dfc-b244-291a8b2a6056</t>
+          <t>embed.imajize.com/915605280?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Sonora-Perfect-Fit-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D2120-24075559/</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sonora Perfect Fit Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/EN/BE1D2120_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/85/BE1D2120_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/8E/BE1D2120_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/T7/BE1D2120_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/211338309?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Olivetta-Tapered-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D3289-23785348/</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Olivetta Tapered Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/ZB/BE1D3289_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/8F/BE1D3289_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/DF/BE1D3289_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/RI/BE1D3289_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/537751906?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Rhiannon-Diamond-Ring-with-Hidden-Accents-Rose-Gold-BE1D6530-17836054/</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Rhiannon Diamond Engagement Ring with Hidden Accents</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/AJ/BE1D6530_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/product_images/FZ/BE1D6530_RG_850px.jpg, https://image.brilliantearth.com/media/carat_image/E4/BE1D6530_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/C1/BE1D6530_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/IS/BE1D6530_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/2873364?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Freesia-Six-Prong-Solitaire-Ring-Rose-Gold-BE1347-21663828/</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Freesia Six-Prong Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/US/BE1347_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/IH/BE1347_rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/75/BE1347_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/DC/BE1347_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/E0/BE1347_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/4074513?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Petite-Luxe-Twisted-Vine-Sapphire-and-Diamond-Ring-(1/8-ct.-tw.)-Rose-Gold-BE1M55S-4464400/</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Petite Luxe Twisted Vine Sapphire and Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/JW/BE1M55S_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/19/BE1M55S_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/50/BE1M55S_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/07/BE1M55S_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/1K/BE1M55S_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/9795267?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Stella-Diamond-Ring-Rose-Gold-BE1D3651-8671632/</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Stella Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/9Z/BE1D3651_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/product_images/AC/BE1D3651_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/0F/BE1D3651_PE_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/CB/BE1D3651_PE_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/4T/BE1D3651_rose_Pear_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/684602870?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Verbena-Diamond-Ring-Rose-Gold-BE1D5481-9424224/</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Verbena Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/G3/BE1D5481_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/2F/BE1D5481_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/TS/BE1D5481_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/BD/BE1D5481_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/A7/BE1D5481_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/GH/BE1D5481_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/852366814?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Bianca-Split-Shank-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D8948-17410572/</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bianca Split Shank Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/3M/BE1D8948_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/DF/BE1D8948_PS_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/4D/BE1D8948_PS_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/S8/BE1D8948_rose_Pear_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/139177022?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Margot-Bezel-Ring-Rose-Gold-BE1D27B5-9519364/</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Margot Bezel Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/XL/BE1D27B5_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/4A/BE1D27B5_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/4E/BE1D27B5_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/AA/BE1D27B5_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/FG/BE1D27B5_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/985657841?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Symphony-Double-Prong-Three-Stone-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D2289-27137785/</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Symphony Double Prong Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Z2/BE1D2289_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/DF/BE1D2289_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/66/BE1D2289_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/P2/BE1D2289_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/220955807?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Freesia-2.7mm-Solitaire-Ring-Rose-Gold-BE1353-23785353/</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Freesia 2.7mm Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/JO/BE1353_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/76/BE1353_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/94/BE1353_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/SY/BE1353_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/747684674?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Melody-Diamond-Ring-Rose-Gold-BE1D6271-9613646/</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Melody Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/K6/BE1D6271_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/89/BE1D6271_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/0R/BE1D6271_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/86/BE1D6271_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/51/BE1D6271_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/2K/BE1D6271_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/707651891?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Comfort-Fit-3mm-Ring-Rose-Gold-BE103-1151344/</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Comfort Fit 3mm Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/NQ/BE103_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/BM/BE103-rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/97/BE103_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/C5/BE103_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/K5/BE103_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/824806323?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Daphne-Art-Deco-Ring-Rose-Gold-BE1DTB150-18041101/</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Daphne Art Deco Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/70/BE1DTB150_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/B3/BE1DTB150_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2D/BE1DTB150_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/BM/BE1DTB150_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/339828721?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Secret-Garden-Lab-Emerald-and-Diamond-Ring-Rose-Gold-BE1LCE6352-21520780/</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Luxe Secret Garden Lab Emerald and Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/BC/BE1LCE6352_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/MR/BE1LCE6352_rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/B8/BE1LCE6352_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2F/BE1LCE6352_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/LP/BE1LCE6352_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/5210286?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Marseille-Halo-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D2011-6306103/</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Marseille Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/54/BE1D2011_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/F5/BE1D2011_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/EC/BE1D2011_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2B/BE1D2011_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/C6/BE1D2011_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/958625076?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Parker-Solitaire-Ring-Rose-Gold-BE1415-15311682/</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Parker Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/2O/BE1415_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/47/BE1415_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/41/BE1415_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/6Z/BE1415_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/202665582?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Viridian-Toi-et-Moi-Diamond-Ring-Rose-Gold-BE1LCE500-16843264/</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Viridian Toi et Moi Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/base_product_center_diamond_images/DY/BE1LCE500_ToiMoi_PearAccent_Emerald_rose_carat_2.jpg, https://image.brilliantearth.com/media/product_images/2F/BE1LCE500_rose_side.jpg, https://image.brilliantearth.com/media/base_product_center_diamond_images/LD/BE1LCE500_ToiMoi_PearAccent_Emerald_rose_carat_2_hd_zo.png</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/252619330?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Horizontal-Petite-Comfort-Fit-Solitaire-Ring-Rose-Gold-BE1815-5245562/</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Horizontal Petite Comfort Fit Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/base_product_center_diamond_images/HT/BE1815_horizontalpeg_Emerald_rose_carat_2.jpg, https://image.brilliantearth.com/media/product_images/4L/BE1815_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/A9/20201021_WG_horizontal_petite_comfort_fit_ER_emerald_diamond_WG_portico_WB_model_on_hand_set_solitaire_accents_crop_1X1_in_house_image.jpg, https://image.brilliantearth.com/media/product_images/T6/BE1815_emerald_rose_side.jpg, https://image.brilliantearth.com/media/base_product_center_diamond_images/AM/BE1815_horizontalpeg_Emerald_rose_carat_2_hd_zo.png</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/7101470?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Olivetta-Diamond-Ring-Rose-Gold-BE1D15103-17281909/</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Olivetta Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/FI/BE1D15103_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/16/BE1D15103_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/14/BE1D15103_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/R2/BE1D15103_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/742324448?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Three-Stone-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1DT2668-10982710/</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Elodie-Cathedral-Diamond-Ring-Rose-Gold-BE1D761-25886005/</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Elodie Cathedral Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/79/BE1D761_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/E8/BE1D761_rose_F_model.JPG, https://image.brilliantearth.com/media/carat_image/5A/BE1D761_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/5D/BE1D761_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/JD/BE1D761_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/796185597?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Nova-Halo-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D25241-1517749/</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Nova Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/IH/BE1D25241_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/FE/BE1D25241_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/JV/BE1D25241_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/AA/BE1D25241_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2B/BE1D25241_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/I8/BE1D25241_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/457874387?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Twisted-Vine-Three-Stone-Diamond-Ring-Rose-Gold-BE1D561-21700303/</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Twisted Vine Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/AO/BE1D561_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/IB/BE1D561_rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/68/BE1D561_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/A1/BE1D561_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/VU/BE1D561_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/1028019?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Entwined-Diamond-Ring-Rose-Gold-BE1D128-26441668/</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Entwined Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/39/BE1D128_rose_Radiant_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/4A/BE1D128_RA_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/46/BE1D128_RA_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/VS/BE1D128_rose_Radiant_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/949011144?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Ballad-Hidden-Floral-Halo-Diamond-Ring-Rose-Gold-BE1D6745-19657221/</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Ballad Hidden Floral Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/KQ/BE1D6745_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_images/3B/BE1D6745LC-rose_020.jpg, https://image.brilliantearth.com/media/carat_image/99/BE1D6745_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E5/BE1D6745_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/4K/BE1D6745_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/7614127?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tacori-Lunetta-Crescent-Cathedral-Diamond-Ring-Rose-Gold-BE1DT2721-20226577/</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tressa-Split-Shank-Diamond-Ring-Rose-Gold-BE1D2014-15417456/</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Tressa Split Shank Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/CS/BE1D2014_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/C9/BE1D2014_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/E8/BE1D2014_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/A7/BE1D2014_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/LT/BE1D2014_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/116401866?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Delicate-Drape-Diamond-Ring-Rose-Gold-BE1DT2682-12921108/</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Melody-Diamond-Ring-(1/5-ct.-tw.)-Rose-Gold-BE1D2299-18973090/</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Luxe Melody Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/GE/BE1D2299_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/61/BE1D2299_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/CE/BE1D2299_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B4/BE1D2299_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/H7/BE1D2299_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/496628172?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Bliss-Diamond-Ring-Rose-Gold-BE1D6541-18137913/</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Bliss Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/FE/BE1D6541_rose_Radiant_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/1F/BE1D6541_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/42/BE1D6541_RA_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B8/BE1D6541_RA_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/TY/BE1D6541_rose_Radiant_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/623938868?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Indigo-Melody-Ring-Rose-Gold-BE1AQ6271-13732432/</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Indigo Melody Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/2Q/BE1AQ6271_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/5A/BE1AQ6271_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/F5/BE1AQ6271_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/87/BE1AQ6271_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/Y1/BE1AQ6271_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/440873711?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Adorned-Camellia-Milgrain-Diamond-Ring-Rose-Gold-BE1D2235-20731212/</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Adorned Camellia Milgrain Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/I2/BE1D2235_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/86/BE1D2235_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/82/BE1D2235_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/8A/BE1D2235_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/LS/BE1D2235_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/2872096?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Cleo-Five-Stone-Diamond-Ring-Rose-Gold-BE1D2233-20731202/</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Cleo Five Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/I9/BE1D2233_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/77/BE1D2233_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/95/BE1D2233_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/EP/BE1D2233_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/3856729?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Adorned-Odessa-Halo-Diamond-Ring-Rose-Gold-BE1D81113-12776476/</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Adorned Odessa Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/S4/BE1D81113_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/B2/BE1D81113_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/97/BE1D81113_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/PR/BE1D81113_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/905516798?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Liliana-Diamond-Ring-Rose-Gold-BE1D2615-17649324/</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Liliana Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Q0/BE1D2615_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/7F/BE1D2615_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/7F/BE1D2615_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/1Q/BE1D2615_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/143021007?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Poetica-Diamond-Ring-Rose-Gold-BE1D2903-19735113/</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Poetica Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/RV/BE1D2903_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/91/BE1D2903_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/99/BE1D2903_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/AZ/BE1D2903_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/6792754?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Adrian-Solitaire-Ring-Rose-Gold-BE1451-11600548/</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Adrian Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/5Z/BE1451_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/B0/BE1451_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/42/BE1451_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/W5/BE1451_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/352612556?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Aria-Halo-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE1D1428-7606384/</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Luxe Aria Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/ZT/BE1D1428_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_images/61/BE1D1428_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/7E/BE1D1428_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/C8/BE1D1428_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/C6/BE1D1428_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/868323338?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Cathedral-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE1DT2671-10982706/</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Mireille-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE1D8383-18909596/</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Mireille Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/L1/BE1D8383_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/4A/BE1D8383_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/90/BE1D8383_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/LG/BE1D8383_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/776329093?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tacori-Lunetta-Crescent-Diamond-Ring-Rose-Gold-BE1DT2720-20226587/</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tressa-Split-Shank-Solitaire-Ring-Rose-Gold-BE1D9282-19701960/</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Tressa Split Shank Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/WT/BE1D9282_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/FC/BE1D9282_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/C7/BE1D9282_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/6Q/BE1D9282_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/1173698?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Adorned-Dawn-Diamond-Ring-Rose-Gold-BE1D1438-14488332/</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Adorned Dawn Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/4P/BE1D1438_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/64/BE1D1438_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/F7/BE1D1438_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B7/BE1D1438_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/7H/BE1D1438_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/3238060?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Dulce-Double-Claw-Prong-Solitaire-Ring-Rose-Gold-BE1D10422-20195171/</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Dulce Double Claw Prong Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/W0/BE1D10422_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/6E/BE1D10422_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/B3/BE1D10422_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/XD/BE1D10422_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/4480489?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Delicate-Aimee-Diamond-Ring-Rose-Gold-BE1D7549-21183498/</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Delicate Aimee Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/DI/BE1D7549_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/D7/BE1D7549_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/E2/BE1D7549_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/BB/BE1D7549_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/26/BE1D7549_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/2404567?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Rhiannon-Three-Stone-Sapphire-Ring-Rose-Gold-BE1S7789-20731248/</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Luxe Rhiannon Three Stone Sapphire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/TS/BE1S7789_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/51/BE1S7789_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/5F/BE1S7789_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/H3/BE1S7789_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/9909881?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Morgan-East-West-Solitaire-Ring-Rose-Gold-BE1943-20901396/</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Morgan East-West Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/shape_images/cd18cb4426d1c44a5976060b289c98f3_3951f629a9744f037a68727055a0c75e_0_.jpg, https://image.brilliantearth.com/media/product_images/JV/BE1943_rose_side.jpg, https://image.brilliantearth.com/media/product_images/WR/BE1943_rose_hand_zo.png</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/849569960?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Freesia-Triple-Prong-Solitaire-Ring-Rose-Gold-BE16412-20194534/</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Freesia Triple-Prong Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/SQ/BE16412_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/8E/BE16412_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/73/BE16412_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/PB/BE16412_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/1619227?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Comfort-Fit-2.5mm-Ring-Rose-Gold-BE1500-2657396/</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Comfort Fit 2.5mm Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/OU/BE1500_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/05/BE1500_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/5B/BE1500_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/NC/BE1500_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/963518784?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Aimee-Three-Stone-Diamond-Ring-Rose-Gold-BE1D647-25467342/</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Aimee Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/TK/BE1D647_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/98/BE1D647_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/91/BE1D647_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/M6/BE1D647_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/424003524?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Willow-Lab-Emerald-and-Diamond-Ring-(1/8-ct.-tw.)-Rose-Gold-BE1LCE1548-21932662/</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Luxe Willow Lab Emerald and Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Z0/BE1LCE1548_rose_Cushion_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/BD/BE1LCE1548_CU_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F5/BE1LCE1548_CU_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/BD/BE1LCE1548_rose_Cushion_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/5911834?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Callista-Diamond-Ring-Rose-Gold-BE1D3975-17564638/</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Callista Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/PB/BE1D3975_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/8F/BE1D3975_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/63/BE1D3975_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/L3/BE1D3975_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/6688697?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Heritage-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D1841-10456706/</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Heritage Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/WV/BE1D1841_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/PY/Luxe-heritage-er--eb.jpg, https://image.brilliantearth.com/media/carat_image/7C/BE1D1841_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E4/BE1D1841_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/56/BE1D1841_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/732079965?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Opera-Accented-Three-Stone-Diamond-Ring-Rose-Gold-BE1D5353-20731217/</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Opera Accented Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/13/BE1D5353_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/27/BE1D5353_PE_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/BB/BE1D5353_PE_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/9S/BE1D5353_rose_Pear_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/6700321?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Quinn-Three-Stone-Diamond-Ring-Rose-Gold-BE1D4257-8598947/</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Quinn Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/I4/BE1D4257_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/C9/BE1D4257_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/9B/BE1D4257_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/2B/BE1D4257_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/E7/BE1D4257_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/3967765?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Alma-Toi-et-Moi-Diamond-Ring-Rose-Gold-BE1D807-11737221/</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Alma Toi et Moi Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/base_product_center_diamond_images/RI/BE1D807_almamoiandtoi_Marquise_rose_carat_2.jpg, https://image.brilliantearth.com/media/product_images/GK/BE1D807_rose_harmony3.jpg, https://image.brilliantearth.com/media/product_images/X5/BE1D807_rose_harmony2.jpg, https://image.brilliantearth.com/media/product_images/NV/BE1D807_rose_side.jpg, https://image.brilliantearth.com/media/product_images/LC/BE1D807_rose_harmony1.jpg, https://image.brilliantearth.com/media/base_product_center_diamond_images/6A/BE1D807_almamoiandtoi_Marquise_rose_carat_2_hd_zo.png</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/5510725?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tacori-Lunetta-Crescent-Three-Stone-Diamond-Ring-Rose-Gold-BE1DT2722-20238001/</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr"/>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Rhiannon-Three-Stone-Lab-Emerald-Ring-Rose-Gold-BE1LCEM1110-22117967/</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Luxe Rhiannon Three Stone Lab Emerald Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/H5/BE1LCEM1110_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/E7/BE1LCEM1110_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F1/BE1LCEM1110_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/BO/BE1LCEM1110_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/451593721?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Joy-Three-Quarter-Coverage-Diamond-Ring-Rose-Gold-BE1D165-15297984/</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Joy Three-Quarter Coverage Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/FI/BE1D165_rose_Cushion_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/17/BE1D165_CU_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/61/BE1D165_CU_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/EA/BE1D165_rose_Cushion_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/962339211?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Luxe-Drape-Diamond-Ring-Rose-Gold-BE1DT2683-12921117/</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr"/>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Petite-Rhiannon-Double-Prong-Three-Stone-Diamond-Ring-Rose-Gold-BE1D1304-21421578/</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Petite Rhiannon Double Prong Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/BA/BE1D1304_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/3D/BE1D1304_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E9/BE1D1304_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/61/BE1D1304_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/2563884?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Delicate-Sienna-Diamond-Ring-Rose-Gold-BE1D2148-24543871/</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Delicate Sienna Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/3E/BE1D2148_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/B2/BE1D2148_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E9/BE1D2148_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/IO/BE1D2148_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tacori-Sculpted-Crescent-Knife-Edge-Diamond-Ring-Rose-Gold-BE1DT2686-12921133/</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Jacinta-Twisting-Split-Shank-Diamond-Ring-Rose-Gold-BE1D6334-19919096/</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Jacinta Twisting Split Shank Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/DO/BE1D6334_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/81/BE1D6334_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/51/BE1D6334_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/0Y/BE1D6334_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/7456898?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Estelle-Halo-Diamond-Ring-(3/4-ct.-tw.)-Rose-Gold-BE1D216-4896694/</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Estelle Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/S3/BE1D216_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_new_images/0D/BE1D216_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/31/BE1D216_rose_additional1.jpg, https://image.brilliantearth.com/media/carat_image/57/BE1D216_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/7A/BE1D216_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/NI/BE1D216_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/618593506?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Baguette-Three-Stone-Diamond-Ring-Rose-Gold-BE1D348-23608706/</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Baguette Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Z8/BE1D348_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/6E/BE1D348_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/1A/BE1D348_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/GU/BE1D348_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/445977924?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Melody-Pavé-Diamond-Ring-Rose-Gold-BE1D6273-23803873/</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Melody Pavé Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/A2/BE1D6273_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/F7/BE1D6273_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/F3/BE1D6273_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/2O/BE1D6273_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/845489091?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Sinclair-Art-Deco-Diamond-Ring-(1/6-ct.-tw.)-Rose-Gold-BE1D1321-16828231/</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Sinclair Art Deco Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/NV/BE1D1321_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/23/BE1D1321_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/FA/BE1D1321_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/9D/BE1D1321_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/334511385?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Jade-Trau-Alure-Solitaire-Ring-Rose-Gold-BE19910-14186694/</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Jade Trau Alure Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/7E/BE19910_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/product_images/WT/JT-6.jpg, https://image.brilliantearth.com/media/carat_image/86/BE19910_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/FF/BE19910_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/FR/BE19910_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/566056344?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tacori-Petite-Crescent-Bloom-Diamond-Ring-Rose-Gold-BE1DTHT2571-10985994/</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tabitha-Channel-Set-Diamond-Ring-Rose-Gold-BE1D117-25847091/</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Tabitha Channel Set Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/CE/BE1D117_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/9B/BE1D117_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/E8/BE1D117_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/HV/BE1D117_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/582680224?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Secret-Garden-Adorned-Gallery-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE1D6561-23468165/</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Secret Garden Adorned Gallery Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/0H/BE1D6561_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/4C/BE1D6561_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/FC/BE1D6561_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/SK/BE1D6561_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/655200012?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Ballad-East-West-Diamond-Ring-Rose-Gold-BE1D18231-20901401/</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Ballad East-West Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/shape_images/51/BE1D18231_emerald_2ct_rose.jpg, https://image.brilliantearth.com/media/product_images/09/BE1D18231_rose_side.jpg, https://image.brilliantearth.com/media/product_images/LY/BE1D18231_rose_hand_zo.png</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/873088937?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Posie-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D8222-20681633/</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Posie Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/XV/BE1D8222_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/08/BE1D8222_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/D4/BE1D8222_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/5A/BE1D8222_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/5908649?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/East-West-Aria-Three-Stone-Diamond-Ring-Rose-Gold-BE1D2321-21926768/</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>East-West Aria Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/shape_images/3f7962a689a8e94568d072fd39013523_d8a89e7b237f03f0489262bb9ba02dcc_0_.jpg, https://image.brilliantearth.com/media/product_images/UE/BE1D2321_rose_side.jpg, https://image.brilliantearth.com/media/product_images/4Z/BE1D2321_rose_hand_zo.png</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/417375641?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Crown-Diamond-Ring-Rose-Gold-BE1DT2650-10982636/</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Tacori-Lunetta-Crescent-Pavé-Three-Stone-Diamond-Ring-Rose-Gold-BE1DT2724-20238011/</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Adorned-Elodie-Perfect-Fit-Diamond-Ring-Rose-Gold-BE1D901-26924416/</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Adorned Elodie Perfect Fit Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/FH/BE1D901_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/EF/BE1D901_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/80/BE1D901_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/YI/BE1D901_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/538109083?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Samara-Eight-Prong-Solitaire-Ring-Rose-Gold-BE19889-19424937/</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Samara Eight-Prong Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/X5/BE19889_rose_Marquise_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/0D/BE19889_MQ_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/87/BE19889_MQ_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/TP/BE19889_rose_Marquise_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/9467508?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Sonnet-Diamond-Ring-Rose-Gold-BE1D7997-22067749/</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Sonnet Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Z2/BE1D7997_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/81/BE1D7997_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/82/BE1D7997_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/5I/BE1D7997_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/5813045?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Princess-Cut-Three-Stone-Diamond-Ring-Rose-Gold-BE1D9800-18909630/</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Princess Cut Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/5I/BE1D9800_rose_Princess_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/25/BE1D9800_PR_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/70/BE1D9800_PR_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/7K/BE1D9800_rose_Princess_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/251177043?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Simply-Tacori-Diamond-Ring-(1/8-ct.-tw.)-Rose-Gold-BE1DT2678-10982632/</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Aimee-Solitaire-Diamond-Ring-with-Hidden-Halo-Rose-Gold-BE1D638-25847081/</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Aimee Solitaire Diamond Engagement Ring with Hidden Halo</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/2N/BE1D638_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/C9/BE1D638_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/EC/BE1D638_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/O7/BE1D638_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/601526191?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Adorned-Luxe-Willow-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D0448-24075579/</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Adorned Luxe Willow Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/LT/BE1D0448_rose_Princess_top_2_carat.png, https://image.brilliantearth.com/media/product_images/6Q/BE1D0448-rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/18/BE1D0448_PR_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/0E/BE1D0448_PR_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/YI/BE1D0448_rose_Princess_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/796056066?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Secret-Garden-Adorned-Gallery-Solitaire-Ring-(1/3-ct.-tw.)-Rose-Gold-BE1D6566-23608712/</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Secret Garden Adorned Gallery Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/GS/BE1D6566_rose_Round_top_75_carat.png, https://image.brilliantearth.com/media/product_images/B2/BE1D6566-rose_F_model.jpg, https://image.brilliantearth.com/media/carat_image/7E/BE1D6566_RD_75ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/C0/BE1D6566_RD_75ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/0R/BE1D6566_rose_Round_hand_zo_50_carat.png</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/654003273?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Soraya-Diamond-Ring-Rose-Gold-BE1D10322-23608717/</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Soraya Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/7I/BE1D10322_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/8B/BE1D10322_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/34/BE1D10322_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/YT/BE1D10322_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/801077184?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Echo-Diamond-Ring-Rose-Gold-BE1D4510-14217291/</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Echo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/2C/BE1D4510_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/74/BE1D4510_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/22/BE1D4510_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/IV/BE1D4510_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/6804320?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Kalina-Hidden-Halo-Diamond-Ring-Rose-Gold-BE1D16192-21650263/</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Kalina Hidden Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/4N/BE1D16192_rose_Radiant_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/A5/BE1D16192_RA_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/48/BE1D16192_RA_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/4G/BE1D16192_rose_Radiant_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/7941782?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Bullet-Shape-Three-Stone-Diamond-Ring-Rose-Gold-BE1D8900-19436947/</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Bullet Shape Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/17/BE1D8900_rose_Pear_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/04/BE1D8900_PE_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/C9/BE1D8900_PE_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/T6/BE1D8900_rose_Pear_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/343991859?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Luxe-Kalina-Hidden-Halo-Diamond-Ring-Rose-Gold-BE1D1825-21752943/</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Luxe Kalina Hidden Halo Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/K7/BE1D1825_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/5F/BE1D1825_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/A5/BE1D1825_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/DN/BE1D1825_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/9870490?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Sloane-Flush-Set-Three-Stone-Diamond-Dome-Ring-Rose-Gold-BE1D993-33371425/</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Sloane Flush Set Three Stone Diamond Dome Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/shape_images/f7e9e9bd894b30338d55245f17564d97_ff31e688da37ecef5ec545c70614181f_0_.png, https://image.brilliantearth.com/media/product_images/FN/BE1D993_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/product_images/4N/BE1D993_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/Y6/BE1D993_OV_200ct_rose_hand_zo.png</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Sloane-Flush-Set-Five-Stone-Diamond-Dome-Ring-Rose-Gold-BE1D994-32751911/</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Sloane Flush Set Five Stone Diamond Dome Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/shape_images/5868b351553e158f1b397ca3418d6a80_ff31e688da37ecef5ec545c70614181f_0_.png, https://image.brilliantearth.com/media/product_images/NS/BE1D994_OV200_rose_side2_old.jpg, https://image.brilliantearth.com/media/product_images/HN/BE1D994_OV200_rose_side1_old.jpg, https://image.brilliantearth.com/media/product_images/47/BE1D994_OV2_rose_hand_zo_old.png</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/758653151?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Julietta-Bezel-Solitaire-Ring-Rose-Gold-BE1798-34777844/</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Julietta Bezel Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/Q9/BE1798_rose_Emerald_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/A5/BE1798_EM_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/3D/BE1798_EM_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/MA/BE1798_rose_Emerald_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/513605108?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Manon-Solitaire-Ring-Rose-Gold-BE1443-35548236/</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Manon Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/H3/BE1443_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/34/BE1443_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/60/BE1443_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/4M/BE1443_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/127219983?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Petite-Fleur-Three-Stone-Diamond-Ring-Rose-Gold-BE1D898-35634836/</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Petite Fleur Three Stone Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/P8/BE1D898_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/11/BE1D898_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/16/BE1D898_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/DB/BE1D898_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/358401600?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Elodie-2.5mm-Solitaire-Ring-Rose-Gold-BE1435-35247771/</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Elodie 2.5mm Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/RE/BE1435_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/D7/BE1435_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/73/BE1435_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/80/BE1435_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/117195357?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Hidden-Heart-Diamond-Ring-Rose-Gold-BE1D326-35372646/</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Hidden Heart Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/2A/BE1D326_rose_Round_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/C2/BE1D326_RD_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/5E/BE1D326_RD_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/HN/BE1D326_rose_Round_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/984668316?v=1739347866</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>https://www.brilliantearth.com/Grand-Versailles-Diamond-Ring-Rose-Gold-BE1D3390-35247776/</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Grand Versailles Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://image.brilliantearth.com/media/diamond_ring_vto/F3/BE1D3390_rose_Oval_top_2_carat.png, https://image.brilliantearth.com/media/carat_image/53/BE1D3390_OV_200ct_rose_side1.jpg, https://image.brilliantearth.com/media/carat_image/00/BE1D3390_OV_200ct_rose_side2.jpg, https://image.brilliantearth.com/media/diamond_ring_vto/KT/BE1D3390_rose_Oval_hand_zo_2_carat.png</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>embed.imajize.com/709787174?v=1739347866</t>
         </is>
       </c>
     </row>

</xml_diff>